<commit_message>
udpate CA E&U and UK prop
</commit_message>
<xml_diff>
--- a/caexcessandumbrella/DataSheet.xlsx
+++ b/caexcessandumbrella/DataSheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://libertymutual-my.sharepoint.com/personal/mohammad_talib_libertymutual_com/Documents/Desktop/regression-pack/caexcessandumbrella/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="6_{F2D74D11-7B77-47B4-A1BC-B9C0C58DB64E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96328848-4EC7-4C45-B546-870A3A66A9A2}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="6_{F2D74D11-7B77-47B4-A1BC-B9C0C58DB64E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DFFB8D06-04EA-4B3E-A59D-6F45E9220CD3}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20250" windowHeight="9150" firstSheet="10" activeTab="12" xr2:uid="{A2EF6AEE-92DE-49D8-BB60-1A120F6353A4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="10" activeTab="12" xr2:uid="{A2EF6AEE-92DE-49D8-BB60-1A120F6353A4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2180" uniqueCount="675">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2181" uniqueCount="679">
   <si>
     <t>First Named Insured</t>
   </si>
@@ -2079,6 +2079,18 @@
   </si>
   <si>
     <t xml:space="preserve">Aon </t>
+  </si>
+  <si>
+    <t>1/1/2026</t>
+  </si>
+  <si>
+    <t>2/1/2026</t>
+  </si>
+  <si>
+    <t>01/01/2026</t>
+  </si>
+  <si>
+    <t>23/10/2026</t>
   </si>
 </sst>
 </file>
@@ -2528,10 +2540,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
@@ -5923,13 +5931,13 @@
         <v>123</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>610</v>
+        <v>675</v>
       </c>
       <c r="K3" t="s">
         <v>428</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>612</v>
+        <v>676</v>
       </c>
       <c r="M3" t="s">
         <v>674</v>
@@ -5988,10 +5996,10 @@
         <v>467</v>
       </c>
       <c r="AG3" s="7" t="s">
-        <v>613</v>
-      </c>
-      <c r="AH3" s="46">
-        <v>46278</v>
+        <v>677</v>
+      </c>
+      <c r="AH3" s="46" t="s">
+        <v>678</v>
       </c>
       <c r="AO3" s="7"/>
       <c r="AZ3" s="7"/>

</xml_diff>